<commit_message>
Apply MT Clinic branding
Green/mint palette with matching dark mode, circle-cross logo with the
MT Clinic / Nursing Care wordmark in the header and on printed quotes,
contact details (phones, Instagram) on quotes and shared text, new app
icons and manifest, RTL-safe rendering for Arabic names, and the
template's example rows taken from the clinic's services card.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NHncMwJnkPWb2bh1MajJ9z
</commit_message>
<xml_diff>
--- a/pricing-template.xlsx
+++ b/pricing-template.xlsx
@@ -39,7 +39,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F5BD8"/>
+      <color rgb="001F7A4F"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -52,7 +52,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F5BD8"/>
+        <fgColor rgb="001F7A4F"/>
       </patternFill>
     </fill>
   </fills>
@@ -452,11 +452,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -505,7 +505,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>GP consultation (20 min)</t>
+          <t>استشارات طبية</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -518,10 +518,12 @@
           <t>visit</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>95</v>
-      </c>
-      <c r="F2" s="2" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Medical consultation</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="b">
         <v>1</v>
       </c>
@@ -529,28 +531,30 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>NUR-01</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Specialist consultation – new patient</t>
+          <t>تعليق مصل</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Consultations</t>
+          <t>Nursing</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F3" s="2" t="n"/>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>IV drip</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="b">
         <v>1</v>
       </c>
@@ -558,28 +562,30 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CON-03</t>
+          <t>NUR-02</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Specialist follow-up</t>
+          <t>إبر بالعضل</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Consultations</t>
+          <t>Nursing</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="F4" s="2" t="n"/>
+          <t>injection</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Intramuscular injection</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="b">
         <v>1</v>
       </c>
@@ -587,28 +593,30 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LAB-01</t>
+          <t>WND-01</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Full blood count</t>
+          <t>قطب جرح (تجميلية)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Wound care</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="F5" s="2" t="n"/>
+          <t>wound</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Wound suturing (cosmetic)</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="b">
         <v>1</v>
       </c>
@@ -616,30 +624,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>LAB-02</t>
+          <t>WND-02</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Comprehensive blood panel</t>
+          <t>تغيير جرح</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Wound care</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>panel</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>199</v>
-      </c>
+          <t>dressing</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>30+ markers</t>
+          <t>Wound dressing change</t>
         </is>
       </c>
       <c r="G6" s="2" t="b">
@@ -649,28 +655,30 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>IMG-01</t>
+          <t>DIA-01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>X-ray – single area</t>
+          <t>تخطيط قلب</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>scan</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>120</v>
-      </c>
-      <c r="F7" s="2" t="n"/>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ECG</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="b">
         <v>1</v>
       </c>
@@ -678,28 +686,30 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IMG-03</t>
+          <t>DIA-02</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MRI – one area</t>
+          <t>فحوصات مخبرية وسحب دم (خدمة منزلية)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>scan</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>450</v>
-      </c>
-      <c r="F8" s="2" t="n"/>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Lab tests &amp; blood draw (home service)</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="b">
         <v>1</v>
       </c>
@@ -707,17 +717,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CAR-01</t>
+          <t>DIA-03</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ECG (12-lead)</t>
+          <t>تحصيل فئات دم</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -725,10 +735,12 @@
           <t>test</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Blood group typing</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="b">
         <v>1</v>
       </c>
@@ -736,30 +748,28 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DER-02</t>
+          <t>SUR-01</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Skin lesion removal</t>
+          <t>علاجات جراحية بسيطة</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Dermatology</t>
+          <t>Minor surgery</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>lesion</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>350</v>
-      </c>
+          <t>procedure</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Histology extra</t>
+          <t>Minor surgical treatment</t>
         </is>
       </c>
       <c r="G10" s="2" t="b">
@@ -769,30 +779,28 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>END-01</t>
+          <t>SUR-02</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Gastroscopy</t>
+          <t>فك جبصين</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Endoscopy</t>
+          <t>Minor surgery</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>procedure</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>1450</v>
-      </c>
+          <t>cast</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sedation included</t>
+          <t>Cast removal</t>
         </is>
       </c>
       <c r="G11" s="2" t="b">
@@ -802,28 +810,30 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>OPH-01</t>
+          <t>SUP-01</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cataract surgery – one eye</t>
+          <t>تأمين لوازم طبية (مشدات، بخار)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Ophthalmology</t>
+          <t>Supplies</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>eye</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>2950</v>
-      </c>
-      <c r="F12" s="2" t="n"/>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Medical supplies (braces, nebulisers)</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="b">
         <v>1</v>
       </c>
@@ -831,28 +841,28 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>OPH-02</t>
+          <t>HOM-01</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Laser eye surgery</t>
+          <t>فرق طبية للخدمة بالمنازل</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Ophthalmology</t>
+          <t>Home care</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>eye</t>
+          <t>visit</t>
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Price on application</t>
+          <t>Home medical team visit</t>
         </is>
       </c>
       <c r="G13" s="2" t="b">
@@ -867,7 +877,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Physiotherapy – initial assessment</t>
+          <t>علاج فيزيائي ومساج</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -880,46 +890,18 @@
           <t>session</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="F14" s="2" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Physiotherapy &amp; massage</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>HLT-01</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Full health check</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Health checks</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>package</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>650</v>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Bloods, ECG, GP review</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="E15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="E16" s="4" t="n"/>
@@ -6887,7 +6869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -6903,74 +6885,81 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>The app reads only the Procedures tab. Blue rows are examples — overwrite or delete them. Keep row 1 (the headers) and the tab name.</t>
+          <t>The app reads only the Procedures tab. Blue rows are examples from the MT Clinic services card — add your prices in column E (blank shows POA), then edit or delete rows. Keep row 1 (the headers) and the tab name.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Names and notes can be in Arabic or English.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>code — short unique ID (e.g. CON-01). Optional but recommended.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>name — what the procedure is called. category — groups the list and creates the filter buttons.</t>
+          <t>code — short unique ID (e.g. CON-01). Optional but recommended.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>unit — shown as “per visit”, “per scan”… (optional).</t>
+          <t>name — what the procedure is called. category — groups the list and creates the filter buttons.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>price — in the currency set in config.js. £1,250.00 or 1250 both work. Leave BLANK to show POA (price on application).</t>
+          <t>unit — shown as “per visit”, “per scan”… (optional).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>price — in the currency set in config.js. £1,250.00 or 1250 both work. Leave BLANK to show POA (price on application).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>notes — shown under the name (optional). active — FALSE / no hides the row; blank means shown.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Sharing</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Share → General access → "Anyone with the link" → Viewer. Only people you add as editors can change prices.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Share → General access → "Anyone with the link" → Viewer. Only people you add as editors can change prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Privacy: anyone with the link (or the sheet ID inside the public website) can read these prices.</t>
         </is>

</xml_diff>